<commit_message>
BCEU, BIFUBC, BCDTRSTY, BPOIFUFE to 2023 SEDS, bug fixes for MPIiFP, BDCSoCaESoPbIC
</commit_message>
<xml_diff>
--- a/InputData/fuels/MPIiFP/Max Perc Inc in Fuel Production.xlsx
+++ b/InputData/fuels/MPIiFP/Max Perc Inc in Fuel Production.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\RMI\RMI_all_states\CO\fuels\MPIiFP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AB5F4CD5-6A4A-4B2C-934C-A6E1AF729BFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B2E44171-1097-4078-98BA-41176D253402}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="525" yWindow="1275" windowWidth="14235" windowHeight="9960" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -490,7 +490,7 @@
         <v>32</v>
       </c>
       <c r="C1" s="6">
-        <v>45294</v>
+        <v>45824</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -772,106 +772,106 @@
         <v>4</v>
       </c>
       <c r="B3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="C3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="D3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="E3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="F3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="G3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="H3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="I3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="J3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="K3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="L3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="M3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="N3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="O3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="P3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Q3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="R3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="S3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="T3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="U3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="V3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="W3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="X3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Y3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Z3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AA3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AB3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AC3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AD3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AE3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AF3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AG3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AH3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AI3">
-        <v>100</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="4" spans="1:35" x14ac:dyDescent="0.25">
@@ -879,106 +879,106 @@
         <v>5</v>
       </c>
       <c r="B4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="C4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="D4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="E4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="F4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="G4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="H4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="I4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="J4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="K4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="L4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="M4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="N4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="O4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="P4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Q4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="R4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="S4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="T4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="U4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="V4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="W4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="X4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Y4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Z4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AA4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AB4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AC4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AD4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AE4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AF4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AG4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AH4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AI4">
-        <v>100</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="5" spans="1:35" x14ac:dyDescent="0.25">
@@ -986,106 +986,106 @@
         <v>6</v>
       </c>
       <c r="B5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="C5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="D5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="E5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="F5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="G5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="H5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="I5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="J5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="K5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="L5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="M5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="N5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="O5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="P5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Q5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="R5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="S5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="T5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="U5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="V5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="W5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="X5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Y5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Z5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AA5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AB5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AC5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AD5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AE5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AF5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AG5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AH5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AI5">
-        <v>100</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="6" spans="1:35" x14ac:dyDescent="0.25">
@@ -1414,106 +1414,106 @@
         <v>10</v>
       </c>
       <c r="B9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="C9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="D9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="E9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="F9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="G9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="H9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="I9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="J9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="K9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="L9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="M9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="N9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="O9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="P9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Q9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="R9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="S9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="T9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="U9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="V9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="W9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="X9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Y9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Z9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AA9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AB9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AC9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AD9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AE9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AF9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AG9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AH9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AI9">
-        <v>100</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="10" spans="1:35" x14ac:dyDescent="0.25">
@@ -1521,106 +1521,106 @@
         <v>11</v>
       </c>
       <c r="B10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="C10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="D10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="E10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="F10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="G10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="H10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="I10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="J10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="K10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="L10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="M10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="N10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="O10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="P10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Q10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="R10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="S10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="T10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="U10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="V10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="W10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="X10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Y10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Z10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AA10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AB10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AC10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AD10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AE10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AF10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AG10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AH10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AI10">
-        <v>100</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="11" spans="1:35" x14ac:dyDescent="0.25">
@@ -1628,106 +1628,106 @@
         <v>12</v>
       </c>
       <c r="B11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="C11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="D11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="E11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="F11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="G11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="H11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="I11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="J11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="K11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="L11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="M11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="N11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="O11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="P11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Q11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="R11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="S11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="T11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="U11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="V11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="W11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="X11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Y11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Z11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AA11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AB11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AC11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AD11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AE11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AF11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AG11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AH11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AI11">
-        <v>100</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="12" spans="1:35" x14ac:dyDescent="0.25">
@@ -1735,106 +1735,106 @@
         <v>13</v>
       </c>
       <c r="B12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="C12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="D12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="E12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="F12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="G12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="H12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="I12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="J12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="K12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="L12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="M12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="N12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="O12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="P12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Q12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="R12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="S12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="T12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="U12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="V12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="W12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="X12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Y12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Z12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AA12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AB12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AC12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AD12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AE12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AF12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AG12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AH12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AI12">
-        <v>100</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="13" spans="1:35" x14ac:dyDescent="0.25">
@@ -1842,106 +1842,106 @@
         <v>14</v>
       </c>
       <c r="B13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="C13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="D13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="E13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="F13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="G13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="H13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="I13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="J13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="K13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="L13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="M13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="N13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="O13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="P13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Q13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="R13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="S13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="T13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="U13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="V13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="W13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="X13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Y13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Z13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AA13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AB13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AC13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AD13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AE13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AF13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AG13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AH13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AI13">
-        <v>100</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.25">
@@ -1949,106 +1949,106 @@
         <v>15</v>
       </c>
       <c r="B14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="C14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="D14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="E14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="F14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="G14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="H14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="I14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="J14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="K14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="L14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="M14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="N14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="O14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="P14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Q14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="R14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="S14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="T14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="U14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="V14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="W14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="X14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Y14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Z14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AA14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AB14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AC14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AD14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AE14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AF14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AG14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AH14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AI14">
-        <v>100</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.25">
@@ -2270,106 +2270,106 @@
         <v>18</v>
       </c>
       <c r="B17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="C17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="D17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="E17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="F17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="G17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="H17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="I17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="J17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="K17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="L17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="M17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="N17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="O17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="P17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Q17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="R17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="S17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="T17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="U17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="V17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="W17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="X17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Y17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Z17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AA17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AB17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AC17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AD17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AE17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AF17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AG17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AH17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AI17">
-        <v>100</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="18" spans="1:35" x14ac:dyDescent="0.25">
@@ -2377,106 +2377,106 @@
         <v>19</v>
       </c>
       <c r="B18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="C18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="D18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="E18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="F18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="G18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="H18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="I18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="J18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="K18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="L18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="M18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="N18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="O18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="P18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Q18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="R18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="S18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="T18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="U18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="V18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="W18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="X18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Y18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Z18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AA18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AB18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AC18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AD18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AE18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AF18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AG18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AH18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AI18">
-        <v>100</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="19" spans="1:35" x14ac:dyDescent="0.25">
@@ -2484,106 +2484,106 @@
         <v>20</v>
       </c>
       <c r="B19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="C19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="D19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="E19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="F19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="G19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="H19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="I19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="J19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="K19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="L19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="M19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="N19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="O19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="P19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Q19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="R19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="S19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="T19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="U19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="V19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="W19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="X19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Y19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Z19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AA19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AB19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AC19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AD19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AE19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AF19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AG19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AH19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AI19">
-        <v>100</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="20" spans="1:35" x14ac:dyDescent="0.25">
@@ -2591,106 +2591,106 @@
         <v>21</v>
       </c>
       <c r="B20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="C20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="D20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="E20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="F20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="G20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="H20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="I20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="J20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="K20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="L20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="M20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="N20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="O20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="P20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Q20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="R20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="S20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="T20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="U20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="V20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="W20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="X20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Y20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Z20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AA20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AB20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AC20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AD20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AE20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AF20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AG20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AH20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AI20">
-        <v>100</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="21" spans="1:35" x14ac:dyDescent="0.25">
@@ -2698,106 +2698,106 @@
         <v>22</v>
       </c>
       <c r="B21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="C21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="D21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="E21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="F21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="G21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="H21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="I21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="J21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="K21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="L21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="M21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="N21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="O21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="P21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Q21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="R21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="S21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="T21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="U21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="V21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="W21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="X21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Y21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Z21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AA21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AB21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AC21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AD21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AE21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AF21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AG21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AH21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AI21">
-        <v>100</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="22" spans="1:35" x14ac:dyDescent="0.25">
@@ -2805,106 +2805,106 @@
         <v>23</v>
       </c>
       <c r="B22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="C22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="D22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="E22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="F22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="G22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="H22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="I22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="J22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="K22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="L22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="M22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="N22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="O22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="P22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Q22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="R22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="S22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="T22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="U22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="V22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="W22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="X22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Y22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="Z22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AA22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AB22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AC22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AD22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AE22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AF22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AG22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AH22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="AI22">
-        <v>100</v>
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>